<commit_message>
feb 28 2nd changes
</commit_message>
<xml_diff>
--- a/TestData/TMTT0005221_StartButtonFunctionalities.xlsx
+++ b/TestData/TMTT0005221_StartButtonFunctionalities.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vijay.kumar\source\repos\SalesForce_Project\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCC8E1E8-0031-4885-8B32-31DA6A73E440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2E7E2F7-4ED2-470D-8BCF-D7CB25162256}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="8" r:id="rId1"/>
@@ -787,14 +787,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -807,14 +807,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -828,14 +828,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="49.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="49.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
@@ -843,7 +843,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -863,9 +863,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -873,7 +873,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>11</v>
       </c>
@@ -889,9 +889,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -899,7 +899,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>11</v>
       </c>
@@ -915,17 +915,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.88671875" customWidth="1"/>
+    <col min="1" max="1" width="27.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>

</xml_diff>